<commit_message>
subiendo primeras cosas de julio
</commit_message>
<xml_diff>
--- a/2026/GALERIA MITRE/Junio/Junio MITRE.xlsx
+++ b/2026/GALERIA MITRE/Junio/Junio MITRE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\2026\GALERIA MITRE\Junio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D846D8-46D4-4D02-94C9-4BC8B06DC054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0417D70-2E5F-44D2-8BD5-07AFB0ED6F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="793" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="199">
   <si>
     <t>TOTAL SUELDO</t>
   </si>
@@ -620,6 +620,12 @@
   </si>
   <si>
     <t>Deposito  $ 112.000,00 abonado el día 08 de julio de 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> local 16 Atanes mikaela Galería Monumenta pago $170.000 20/07</t>
+  </si>
+  <si>
+    <t>L 16</t>
   </si>
 </sst>
 </file>
@@ -802,7 +808,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -884,6 +890,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1247,7 +1259,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="218">
+  <cellXfs count="223">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1481,145 +1493,150 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -2046,7 +2063,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="63"/>
-      <c r="B9" s="172" t="s">
+      <c r="B9" s="182" t="s">
         <v>166</v>
       </c>
       <c r="C9" s="63"/>
@@ -2054,13 +2071,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="63"/>
-      <c r="B10" s="172"/>
+      <c r="B10" s="182"/>
       <c r="C10" s="63"/>
       <c r="D10" s="63"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="63"/>
-      <c r="B11" s="172"/>
+      <c r="B11" s="182"/>
       <c r="C11" s="63"/>
       <c r="D11" s="63"/>
     </row>
@@ -2143,10 +2160,10 @@
       <c r="F22" s="129"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="170" t="s">
+      <c r="A23" s="177" t="s">
         <v>167</v>
       </c>
-      <c r="B23" s="171"/>
+      <c r="B23" s="178"/>
       <c r="C23" s="82">
         <v>1231605.7</v>
       </c>
@@ -2193,10 +2210,10 @@
       <c r="F26" s="129"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="170" t="s">
+      <c r="A27" s="177" t="s">
         <v>168</v>
       </c>
-      <c r="B27" s="171"/>
+      <c r="B27" s="178"/>
       <c r="C27" s="82">
         <v>815681.8</v>
       </c>
@@ -2285,10 +2302,10 @@
       <c r="F35" s="4"/>
     </row>
     <row r="36" spans="1:7" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="170" t="s">
+      <c r="A36" s="177" t="s">
         <v>183</v>
       </c>
-      <c r="B36" s="171"/>
+      <c r="B36" s="178"/>
       <c r="C36" s="82">
         <v>710000</v>
       </c>
@@ -2341,10 +2358,10 @@
       <c r="D40" s="31"/>
     </row>
     <row r="41" spans="1:7" s="19" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="170" t="s">
+      <c r="A41" s="177" t="s">
         <v>130</v>
       </c>
-      <c r="B41" s="171"/>
+      <c r="B41" s="178"/>
       <c r="C41" s="96">
         <v>111379</v>
       </c>
@@ -2383,10 +2400,10 @@
       <c r="F44" s="74"/>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="170" t="s">
+      <c r="A45" s="177" t="s">
         <v>181</v>
       </c>
-      <c r="B45" s="171"/>
+      <c r="B45" s="178"/>
       <c r="C45" s="100">
         <v>11596.99</v>
       </c>
@@ -2396,10 +2413,10 @@
       <c r="F45" s="74"/>
     </row>
     <row r="46" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="170" t="s">
+      <c r="A46" s="177" t="s">
         <v>129</v>
       </c>
-      <c r="B46" s="171"/>
+      <c r="B46" s="178"/>
       <c r="C46" s="100">
         <v>11930.96</v>
       </c>
@@ -2552,10 +2569,10 @@
       <c r="D58" s="55"/>
     </row>
     <row r="59" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="177" t="s">
+      <c r="A59" s="179" t="s">
         <v>156</v>
       </c>
-      <c r="B59" s="178"/>
+      <c r="B59" s="180"/>
       <c r="C59" s="85">
         <v>202000</v>
       </c>
@@ -2564,10 +2581,10 @@
       </c>
     </row>
     <row r="60" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="177" t="s">
+      <c r="A60" s="179" t="s">
         <v>176</v>
       </c>
-      <c r="B60" s="178"/>
+      <c r="B60" s="180"/>
       <c r="C60" s="85">
         <v>229900</v>
       </c>
@@ -2576,10 +2593,10 @@
       </c>
     </row>
     <row r="61" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="170" t="s">
+      <c r="A61" s="177" t="s">
         <v>178</v>
       </c>
-      <c r="B61" s="171"/>
+      <c r="B61" s="178"/>
       <c r="C61" s="85">
         <v>35000</v>
       </c>
@@ -2590,10 +2607,10 @@
       <c r="F61" s="24"/>
     </row>
     <row r="62" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="177" t="s">
+      <c r="A62" s="179" t="s">
         <v>179</v>
       </c>
-      <c r="B62" s="178"/>
+      <c r="B62" s="180"/>
       <c r="C62" s="85">
         <v>9395</v>
       </c>
@@ -2607,10 +2624,10 @@
       <c r="F62" s="24"/>
     </row>
     <row r="63" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="177" t="s">
+      <c r="A63" s="179" t="s">
         <v>171</v>
       </c>
-      <c r="B63" s="178"/>
+      <c r="B63" s="180"/>
       <c r="C63" s="85">
         <v>18300</v>
       </c>
@@ -2668,10 +2685,10 @@
       <c r="D67" s="55"/>
     </row>
     <row r="68" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="170" t="s">
+      <c r="A68" s="177" t="s">
         <v>73</v>
       </c>
-      <c r="B68" s="171"/>
+      <c r="B68" s="178"/>
       <c r="C68" s="85">
         <v>60000</v>
       </c>
@@ -2758,14 +2775,14 @@
       <c r="D77" s="68"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="170"/>
-      <c r="B78" s="171"/>
+      <c r="A78" s="177"/>
+      <c r="B78" s="178"/>
       <c r="C78" s="56"/>
       <c r="D78" s="54"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="170"/>
-      <c r="B79" s="171"/>
+      <c r="A79" s="177"/>
+      <c r="B79" s="178"/>
       <c r="C79" s="56"/>
       <c r="D79" s="54"/>
     </row>
@@ -2981,14 +2998,14 @@
       <c r="D108" s="99"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A109" s="169" t="s">
+      <c r="A109" s="181" t="s">
         <v>50</v>
       </c>
-      <c r="B109" s="169"/>
+      <c r="B109" s="181"/>
     </row>
     <row r="110" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="169"/>
-      <c r="B110" s="169"/>
+      <c r="A110" s="181"/>
+      <c r="B110" s="181"/>
     </row>
     <row r="111" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="69" t="s">
@@ -3028,6 +3045,12 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A109:B110"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A36:B36"/>
     <mergeCell ref="A4:B7"/>
     <mergeCell ref="A14:D17"/>
     <mergeCell ref="A72:C72"/>
@@ -3041,12 +3064,6 @@
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A109:B110"/>
-    <mergeCell ref="A79:B79"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A36:B36"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3081,17 +3098,17 @@
   <sheetData>
     <row r="1" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
-      <c r="B1" s="185" t="s">
+      <c r="B1" s="183" t="s">
         <v>151</v>
       </c>
-      <c r="C1" s="186"/>
-      <c r="D1" s="186"/>
-      <c r="E1" s="186"/>
-      <c r="F1" s="186"/>
-      <c r="G1" s="186"/>
-      <c r="H1" s="186"/>
-      <c r="I1" s="186"/>
-      <c r="J1" s="187"/>
+      <c r="C1" s="184"/>
+      <c r="D1" s="184"/>
+      <c r="E1" s="184"/>
+      <c r="F1" s="184"/>
+      <c r="G1" s="184"/>
+      <c r="H1" s="184"/>
+      <c r="I1" s="184"/>
+      <c r="J1" s="185"/>
       <c r="K1" s="111" t="s">
         <v>4</v>
       </c>
@@ -3109,15 +3126,15 @@
     </row>
     <row r="2" spans="1:18" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
-      <c r="B2" s="188"/>
-      <c r="C2" s="189"/>
-      <c r="D2" s="189"/>
-      <c r="E2" s="189"/>
-      <c r="F2" s="189"/>
-      <c r="G2" s="189"/>
-      <c r="H2" s="189"/>
-      <c r="I2" s="189"/>
-      <c r="J2" s="190"/>
+      <c r="B2" s="186"/>
+      <c r="C2" s="187"/>
+      <c r="D2" s="187"/>
+      <c r="E2" s="187"/>
+      <c r="F2" s="187"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="187"/>
+      <c r="J2" s="188"/>
       <c r="K2" s="113" t="s">
         <v>63</v>
       </c>
@@ -3148,40 +3165,40 @@
       <c r="O3" s="204"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4" s="179" t="s">
+      <c r="A4" s="205" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="181" t="s">
+      <c r="B4" s="207" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="183" t="s">
+      <c r="C4" s="192" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="183" t="s">
+      <c r="D4" s="192" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="183" t="s">
+      <c r="E4" s="192" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="183" t="s">
+      <c r="F4" s="192" t="s">
         <v>60</v>
       </c>
-      <c r="G4" s="183" t="s">
+      <c r="G4" s="192" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="183" t="s">
+      <c r="H4" s="192" t="s">
         <v>47</v>
       </c>
       <c r="I4" s="197" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="195" t="s">
+      <c r="J4" s="194" t="s">
         <v>46</v>
       </c>
-      <c r="K4" s="195" t="s">
+      <c r="K4" s="194" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="195" t="s">
+      <c r="L4" s="194" t="s">
         <v>45</v>
       </c>
       <c r="M4" s="200" t="s">
@@ -3190,30 +3207,30 @@
       <c r="N4" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="O4" s="191" t="s">
+      <c r="O4" s="189" t="s">
         <v>56</v>
       </c>
       <c r="R4" s="24"/>
     </row>
     <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="180"/>
-      <c r="B5" s="182"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
-      <c r="E5" s="184"/>
-      <c r="F5" s="184"/>
-      <c r="G5" s="184"/>
-      <c r="H5" s="194"/>
+      <c r="A5" s="206"/>
+      <c r="B5" s="208"/>
+      <c r="C5" s="196"/>
+      <c r="D5" s="196"/>
+      <c r="E5" s="196"/>
+      <c r="F5" s="196"/>
+      <c r="G5" s="196"/>
+      <c r="H5" s="193"/>
       <c r="I5" s="198"/>
-      <c r="J5" s="196"/>
+      <c r="J5" s="195"/>
       <c r="K5" s="199"/>
-      <c r="L5" s="196"/>
+      <c r="L5" s="195"/>
       <c r="M5" s="201"/>
       <c r="N5" s="28" t="str">
         <f>RESUMEN!B9</f>
         <v>VTO 17/07</v>
       </c>
-      <c r="O5" s="192"/>
+      <c r="O5" s="190"/>
     </row>
     <row r="6" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="130" t="s">
@@ -4122,14 +4139,14 @@
     </row>
     <row r="22" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="130"/>
-      <c r="B22" s="87">
+      <c r="B22" s="222">
         <f t="shared" si="6"/>
         <v>16</v>
       </c>
-      <c r="C22" s="87" t="s">
+      <c r="C22" s="222" t="s">
         <v>118</v>
       </c>
-      <c r="D22" s="87" t="s">
+      <c r="D22" s="222" t="s">
         <v>87</v>
       </c>
       <c r="E22" s="32">
@@ -5564,14 +5581,14 @@
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" s="74"/>
-      <c r="B47" s="214">
+      <c r="B47" s="169">
         <f t="shared" si="8"/>
         <v>41</v>
       </c>
-      <c r="C47" s="214">
+      <c r="C47" s="169">
         <v>3304</v>
       </c>
-      <c r="D47" s="214" t="s">
+      <c r="D47" s="169" t="s">
         <v>131</v>
       </c>
       <c r="E47" s="32">
@@ -6624,87 +6641,92 @@
     </row>
     <row r="68" spans="2:16" hidden="1" x14ac:dyDescent="0.3"/>
     <row r="69" spans="2:16" ht="9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D69" s="193" t="s">
+      <c r="D69" s="191" t="s">
         <v>69</v>
       </c>
-      <c r="E69" s="193"/>
-      <c r="F69" s="193"/>
-      <c r="G69" s="193"/>
-      <c r="H69" s="193"/>
-      <c r="I69" s="193"/>
-      <c r="J69" s="193"/>
-      <c r="K69" s="193"/>
-      <c r="L69" s="193"/>
-      <c r="M69" s="193"/>
-      <c r="N69" s="193"/>
+      <c r="E69" s="191"/>
+      <c r="F69" s="191"/>
+      <c r="G69" s="191"/>
+      <c r="H69" s="191"/>
+      <c r="I69" s="191"/>
+      <c r="J69" s="191"/>
+      <c r="K69" s="191"/>
+      <c r="L69" s="191"/>
+      <c r="M69" s="191"/>
+      <c r="N69" s="191"/>
     </row>
     <row r="70" spans="2:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D70" s="193"/>
-      <c r="E70" s="193"/>
-      <c r="F70" s="193"/>
-      <c r="G70" s="193"/>
-      <c r="H70" s="193"/>
-      <c r="I70" s="193"/>
-      <c r="J70" s="193"/>
-      <c r="K70" s="193"/>
-      <c r="L70" s="193"/>
-      <c r="M70" s="193"/>
-      <c r="N70" s="193"/>
+      <c r="D70" s="191"/>
+      <c r="E70" s="191"/>
+      <c r="F70" s="191"/>
+      <c r="G70" s="191"/>
+      <c r="H70" s="191"/>
+      <c r="I70" s="191"/>
+      <c r="J70" s="191"/>
+      <c r="K70" s="191"/>
+      <c r="L70" s="191"/>
+      <c r="M70" s="191"/>
+      <c r="N70" s="191"/>
     </row>
     <row r="71" spans="2:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D71" s="193"/>
-      <c r="E71" s="193"/>
-      <c r="F71" s="193"/>
-      <c r="G71" s="193"/>
-      <c r="H71" s="193"/>
-      <c r="I71" s="193"/>
-      <c r="J71" s="193"/>
-      <c r="K71" s="193"/>
-      <c r="L71" s="193"/>
-      <c r="M71" s="193"/>
-      <c r="N71" s="193"/>
+      <c r="D71" s="191"/>
+      <c r="E71" s="191"/>
+      <c r="F71" s="191"/>
+      <c r="G71" s="191"/>
+      <c r="H71" s="191"/>
+      <c r="I71" s="191"/>
+      <c r="J71" s="191"/>
+      <c r="K71" s="191"/>
+      <c r="L71" s="191"/>
+      <c r="M71" s="191"/>
+      <c r="N71" s="191"/>
     </row>
     <row r="72" spans="2:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D72" s="193"/>
-      <c r="E72" s="193"/>
-      <c r="F72" s="193"/>
-      <c r="G72" s="193"/>
-      <c r="H72" s="193"/>
-      <c r="I72" s="193"/>
-      <c r="J72" s="193"/>
-      <c r="K72" s="193"/>
-      <c r="L72" s="193"/>
-      <c r="M72" s="193"/>
-      <c r="N72" s="193"/>
+      <c r="D72" s="191"/>
+      <c r="E72" s="191"/>
+      <c r="F72" s="191"/>
+      <c r="G72" s="191"/>
+      <c r="H72" s="191"/>
+      <c r="I72" s="191"/>
+      <c r="J72" s="191"/>
+      <c r="K72" s="191"/>
+      <c r="L72" s="191"/>
+      <c r="M72" s="191"/>
+      <c r="N72" s="191"/>
     </row>
     <row r="73" spans="2:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D73" s="193"/>
-      <c r="E73" s="193"/>
-      <c r="F73" s="193"/>
-      <c r="G73" s="193"/>
-      <c r="H73" s="193"/>
-      <c r="I73" s="193"/>
-      <c r="J73" s="193"/>
-      <c r="K73" s="193"/>
-      <c r="L73" s="193"/>
-      <c r="M73" s="193"/>
-      <c r="N73" s="193"/>
+      <c r="D73" s="191"/>
+      <c r="E73" s="191"/>
+      <c r="F73" s="191"/>
+      <c r="G73" s="191"/>
+      <c r="H73" s="191"/>
+      <c r="I73" s="191"/>
+      <c r="J73" s="191"/>
+      <c r="K73" s="191"/>
+      <c r="L73" s="191"/>
+      <c r="M73" s="191"/>
+      <c r="N73" s="191"/>
     </row>
     <row r="74" spans="2:16" ht="65.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D74" s="193"/>
-      <c r="E74" s="193"/>
-      <c r="F74" s="193"/>
-      <c r="G74" s="193"/>
-      <c r="H74" s="193"/>
-      <c r="I74" s="193"/>
-      <c r="J74" s="193"/>
-      <c r="K74" s="193"/>
-      <c r="L74" s="193"/>
-      <c r="M74" s="193"/>
-      <c r="N74" s="193"/>
+      <c r="D74" s="191"/>
+      <c r="E74" s="191"/>
+      <c r="F74" s="191"/>
+      <c r="G74" s="191"/>
+      <c r="H74" s="191"/>
+      <c r="I74" s="191"/>
+      <c r="J74" s="191"/>
+      <c r="K74" s="191"/>
+      <c r="L74" s="191"/>
+      <c r="M74" s="191"/>
+      <c r="N74" s="191"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
     <mergeCell ref="B1:J2"/>
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="D69:N74"/>
@@ -6717,11 +6739,6 @@
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="M4:M5"/>
     <mergeCell ref="B3:O3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" orientation="landscape" r:id="rId1"/>
@@ -6730,7 +6747,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B56D240-6D8B-4144-A545-69291A6FAA07}">
-  <dimension ref="C2:J32"/>
+  <dimension ref="C2:J40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -6767,34 +6784,34 @@
       <c r="J5" s="23"/>
     </row>
     <row r="6" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C6" s="205" t="s">
+      <c r="C6" s="209" t="s">
         <v>191</v>
       </c>
-      <c r="D6" s="206"/>
-      <c r="E6" s="206"/>
-      <c r="F6" s="206"/>
-      <c r="G6" s="206"/>
-      <c r="H6" s="207"/>
+      <c r="D6" s="210"/>
+      <c r="E6" s="210"/>
+      <c r="F6" s="210"/>
+      <c r="G6" s="210"/>
+      <c r="H6" s="211"/>
       <c r="I6" s="23"/>
       <c r="J6" s="23"/>
     </row>
     <row r="7" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C7" s="208"/>
-      <c r="D7" s="209"/>
-      <c r="E7" s="209"/>
-      <c r="F7" s="209"/>
-      <c r="G7" s="209"/>
-      <c r="H7" s="210"/>
+      <c r="C7" s="212"/>
+      <c r="D7" s="213"/>
+      <c r="E7" s="213"/>
+      <c r="F7" s="213"/>
+      <c r="G7" s="213"/>
+      <c r="H7" s="214"/>
       <c r="I7" s="23"/>
       <c r="J7" s="23"/>
     </row>
     <row r="8" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C8" s="211"/>
-      <c r="D8" s="212"/>
-      <c r="E8" s="212"/>
-      <c r="F8" s="212"/>
-      <c r="G8" s="212"/>
-      <c r="H8" s="213"/>
+      <c r="C8" s="215"/>
+      <c r="D8" s="216"/>
+      <c r="E8" s="216"/>
+      <c r="F8" s="216"/>
+      <c r="G8" s="216"/>
+      <c r="H8" s="217"/>
       <c r="I8" s="74"/>
       <c r="J8" s="74"/>
     </row>
@@ -6834,30 +6851,30 @@
       <c r="H13" s="119"/>
     </row>
     <row r="14" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C14" s="205" t="s">
+      <c r="C14" s="209" t="s">
         <v>194</v>
       </c>
-      <c r="D14" s="206"/>
-      <c r="E14" s="206"/>
-      <c r="F14" s="206"/>
-      <c r="G14" s="206"/>
-      <c r="H14" s="207"/>
+      <c r="D14" s="210"/>
+      <c r="E14" s="210"/>
+      <c r="F14" s="210"/>
+      <c r="G14" s="210"/>
+      <c r="H14" s="211"/>
     </row>
     <row r="15" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C15" s="208"/>
-      <c r="D15" s="209"/>
-      <c r="E15" s="209"/>
-      <c r="F15" s="209"/>
-      <c r="G15" s="209"/>
-      <c r="H15" s="210"/>
+      <c r="C15" s="212"/>
+      <c r="D15" s="213"/>
+      <c r="E15" s="213"/>
+      <c r="F15" s="213"/>
+      <c r="G15" s="213"/>
+      <c r="H15" s="214"/>
     </row>
     <row r="16" spans="3:10" ht="117" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C16" s="211"/>
-      <c r="D16" s="212"/>
-      <c r="E16" s="212"/>
-      <c r="F16" s="212"/>
-      <c r="G16" s="212"/>
-      <c r="H16" s="213"/>
+      <c r="C16" s="215"/>
+      <c r="D16" s="216"/>
+      <c r="E16" s="216"/>
+      <c r="F16" s="216"/>
+      <c r="G16" s="216"/>
+      <c r="H16" s="217"/>
     </row>
     <row r="18" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="19" spans="3:8" x14ac:dyDescent="0.3">
@@ -6888,37 +6905,37 @@
       <c r="H21" s="119"/>
     </row>
     <row r="22" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C22" s="205" t="s">
+      <c r="C22" s="209" t="s">
         <v>195</v>
       </c>
-      <c r="D22" s="206"/>
-      <c r="E22" s="206"/>
-      <c r="F22" s="206"/>
-      <c r="G22" s="206"/>
-      <c r="H22" s="207"/>
+      <c r="D22" s="210"/>
+      <c r="E22" s="210"/>
+      <c r="F22" s="210"/>
+      <c r="G22" s="210"/>
+      <c r="H22" s="211"/>
     </row>
     <row r="23" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C23" s="208"/>
-      <c r="D23" s="209"/>
-      <c r="E23" s="209"/>
-      <c r="F23" s="209"/>
-      <c r="G23" s="209"/>
-      <c r="H23" s="210"/>
+      <c r="C23" s="212"/>
+      <c r="D23" s="213"/>
+      <c r="E23" s="213"/>
+      <c r="F23" s="213"/>
+      <c r="G23" s="213"/>
+      <c r="H23" s="214"/>
     </row>
     <row r="24" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C24" s="211"/>
-      <c r="D24" s="212"/>
-      <c r="E24" s="212"/>
-      <c r="F24" s="212"/>
-      <c r="G24" s="212"/>
-      <c r="H24" s="213"/>
+      <c r="C24" s="215"/>
+      <c r="D24" s="216"/>
+      <c r="E24" s="216"/>
+      <c r="F24" s="216"/>
+      <c r="G24" s="216"/>
+      <c r="H24" s="217"/>
     </row>
     <row r="26" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C27" s="215" t="s">
+      <c r="C27" s="170" t="s">
         <v>154</v>
       </c>
-      <c r="D27" s="216">
+      <c r="D27" s="171">
         <f>D19+1</f>
         <v>4</v>
       </c>
@@ -6928,7 +6945,7 @@
       <c r="H27" s="118"/>
     </row>
     <row r="28" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C28" s="217" t="s">
+      <c r="C28" s="172" t="s">
         <v>155</v>
       </c>
       <c r="D28" s="129">
@@ -6937,42 +6954,97 @@
       <c r="H28" s="119"/>
     </row>
     <row r="29" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C29" s="217"/>
+      <c r="C29" s="172"/>
       <c r="D29" s="129"/>
       <c r="H29" s="119"/>
     </row>
     <row r="30" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C30" s="205" t="s">
+      <c r="C30" s="209" t="s">
         <v>196</v>
       </c>
-      <c r="D30" s="206"/>
-      <c r="E30" s="206"/>
-      <c r="F30" s="206"/>
-      <c r="G30" s="206"/>
-      <c r="H30" s="207"/>
+      <c r="D30" s="210"/>
+      <c r="E30" s="210"/>
+      <c r="F30" s="210"/>
+      <c r="G30" s="210"/>
+      <c r="H30" s="211"/>
     </row>
     <row r="31" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C31" s="208"/>
-      <c r="D31" s="209"/>
-      <c r="E31" s="209"/>
-      <c r="F31" s="209"/>
-      <c r="G31" s="209"/>
-      <c r="H31" s="210"/>
+      <c r="C31" s="212"/>
+      <c r="D31" s="213"/>
+      <c r="E31" s="213"/>
+      <c r="F31" s="213"/>
+      <c r="G31" s="213"/>
+      <c r="H31" s="214"/>
     </row>
     <row r="32" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C32" s="211"/>
-      <c r="D32" s="212"/>
-      <c r="E32" s="212"/>
-      <c r="F32" s="212"/>
-      <c r="G32" s="212"/>
-      <c r="H32" s="213"/>
+      <c r="C32" s="215"/>
+      <c r="D32" s="216"/>
+      <c r="E32" s="216"/>
+      <c r="F32" s="216"/>
+      <c r="G32" s="216"/>
+      <c r="H32" s="217"/>
+    </row>
+    <row r="34" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="35" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C35" s="218" t="s">
+        <v>154</v>
+      </c>
+      <c r="D35" s="219">
+        <f>D27+1</f>
+        <v>5</v>
+      </c>
+      <c r="E35" s="117"/>
+      <c r="F35" s="117"/>
+      <c r="G35" s="117"/>
+      <c r="H35" s="118"/>
+    </row>
+    <row r="36" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C36" s="220" t="s">
+        <v>155</v>
+      </c>
+      <c r="D36" s="221" t="s">
+        <v>198</v>
+      </c>
+      <c r="H36" s="119"/>
+    </row>
+    <row r="37" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C37" s="220"/>
+      <c r="D37" s="221"/>
+      <c r="H37" s="119"/>
+    </row>
+    <row r="38" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C38" s="209" t="s">
+        <v>197</v>
+      </c>
+      <c r="D38" s="210"/>
+      <c r="E38" s="210"/>
+      <c r="F38" s="210"/>
+      <c r="G38" s="210"/>
+      <c r="H38" s="211"/>
+    </row>
+    <row r="39" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C39" s="212"/>
+      <c r="D39" s="213"/>
+      <c r="E39" s="213"/>
+      <c r="F39" s="213"/>
+      <c r="G39" s="213"/>
+      <c r="H39" s="214"/>
+    </row>
+    <row r="40" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C40" s="215"/>
+      <c r="D40" s="216"/>
+      <c r="E40" s="216"/>
+      <c r="F40" s="216"/>
+      <c r="G40" s="216"/>
+      <c r="H40" s="217"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="C6:H8"/>
     <mergeCell ref="C14:H16"/>
     <mergeCell ref="C22:H24"/>
     <mergeCell ref="C30:H32"/>
+    <mergeCell ref="C38:H40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>